<commit_message>
Updated TJK_grids model - 2025-09-25 15:32
</commit_message>
<xml_diff>
--- a/VerveStacks_TJK_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_TJK_grids/ReportDefs_vervestacks.xlsx
@@ -5,30 +5,32 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\VerveStacks\assumptions\VerveStacks_ISO_template\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_TJK_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9080BAB-9E79-43E9-804D-92CCE048C677}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6E2B6A29-FDBB-4CDB-9F23-65D3EE2F7273}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ScenMap_OLD" sheetId="70" r:id="rId1"/>
     <sheet name="ScenMap" sheetId="56" r:id="rId2"/>
-    <sheet name="TS_Defs" sheetId="27" r:id="rId3"/>
-    <sheet name="TS_ratios" sheetId="68" r:id="rId4"/>
-    <sheet name="Sankey" sheetId="69" r:id="rId5"/>
-    <sheet name="PSet_MAP" sheetId="57" r:id="rId6"/>
-    <sheet name="CSET_MAP" sheetId="66" r:id="rId7"/>
-    <sheet name="CName_MAP" sheetId="58" r:id="rId8"/>
-    <sheet name="timeslice map" sheetId="64" r:id="rId9"/>
-    <sheet name="process map" sheetId="65" r:id="rId10"/>
-    <sheet name="commodity map" sheetId="67" r:id="rId11"/>
-    <sheet name="ATS" sheetId="63" r:id="rId12"/>
-    <sheet name="UnitConv" sheetId="59" r:id="rId13"/>
+    <sheet name="geolocation" sheetId="72" r:id="rId3"/>
+    <sheet name="process_map_geo" sheetId="71" r:id="rId4"/>
+    <sheet name="TS_Defs" sheetId="27" r:id="rId5"/>
+    <sheet name="TS_ratios" sheetId="68" r:id="rId6"/>
+    <sheet name="Sankey" sheetId="69" r:id="rId7"/>
+    <sheet name="PSet_MAP" sheetId="57" r:id="rId8"/>
+    <sheet name="CSET_MAP" sheetId="66" r:id="rId9"/>
+    <sheet name="CName_MAP" sheetId="58" r:id="rId10"/>
+    <sheet name="timeslice map" sheetId="64" r:id="rId11"/>
+    <sheet name="process map" sheetId="65" r:id="rId12"/>
+    <sheet name="commodity map" sheetId="67" r:id="rId13"/>
+    <sheet name="ATS" sheetId="63" r:id="rId14"/>
+    <sheet name="UnitConv" sheetId="59" r:id="rId15"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">TS_Defs!$A$2:$N$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">TS_Defs!$A$2:$N$2</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -82,7 +84,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="859" uniqueCount="423">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1187" uniqueCount="526">
   <si>
     <t>Unit</t>
   </si>
@@ -1351,6 +1353,315 @@
   </si>
   <si>
     <t>e[_]*</t>
+  </si>
+  <si>
+    <t>grid_node</t>
+  </si>
+  <si>
+    <t>p_w242159365</t>
+  </si>
+  <si>
+    <t>p_w488077624</t>
+  </si>
+  <si>
+    <t>p_w799346816</t>
+  </si>
+  <si>
+    <t>p_w1016951696</t>
+  </si>
+  <si>
+    <t>p_w1373384046</t>
+  </si>
+  <si>
+    <t>p_TJ6</t>
+  </si>
+  <si>
+    <t>p_TJ29</t>
+  </si>
+  <si>
+    <t>p_TJ20</t>
+  </si>
+  <si>
+    <t>p_TJ46</t>
+  </si>
+  <si>
+    <t>p_TJ30</t>
+  </si>
+  <si>
+    <t>p_TJ4</t>
+  </si>
+  <si>
+    <t>p_TJ10</t>
+  </si>
+  <si>
+    <t>p_TJ26</t>
+  </si>
+  <si>
+    <t>rez_spv_001</t>
+  </si>
+  <si>
+    <t>rez_spv_002</t>
+  </si>
+  <si>
+    <t>rez_spv_003</t>
+  </si>
+  <si>
+    <t>rez_spv_004</t>
+  </si>
+  <si>
+    <t>rez_spv_005</t>
+  </si>
+  <si>
+    <t>rez_spv_006</t>
+  </si>
+  <si>
+    <t>rez_spv_007</t>
+  </si>
+  <si>
+    <t>rez_spv_008</t>
+  </si>
+  <si>
+    <t>rez_spv_009</t>
+  </si>
+  <si>
+    <t>rez_spv_010</t>
+  </si>
+  <si>
+    <t>rez_won_001</t>
+  </si>
+  <si>
+    <t>rez_won_002</t>
+  </si>
+  <si>
+    <t>rez_won_003</t>
+  </si>
+  <si>
+    <t>rez_won_004</t>
+  </si>
+  <si>
+    <t>rez_won_005</t>
+  </si>
+  <si>
+    <t>admin_1</t>
+  </si>
+  <si>
+    <t>Leninabad</t>
+  </si>
+  <si>
+    <t>Tadzhikistan Territories</t>
+  </si>
+  <si>
+    <t>Khatlon</t>
+  </si>
+  <si>
+    <t>Kashkadarya</t>
+  </si>
+  <si>
+    <t>Tashkent</t>
+  </si>
+  <si>
+    <t>Surkhandarya</t>
+  </si>
+  <si>
+    <t>Ferghana</t>
+  </si>
+  <si>
+    <t>Batken</t>
+  </si>
+  <si>
+    <t>Badakhshan</t>
+  </si>
+  <si>
+    <t>Jizzakh</t>
+  </si>
+  <si>
+    <t>Kunduz</t>
+  </si>
+  <si>
+    <t>Sirdaryo</t>
+  </si>
+  <si>
+    <t>region_com</t>
+  </si>
+  <si>
+    <t>e_w242159365-500</t>
+  </si>
+  <si>
+    <t>e_w488077624-500</t>
+  </si>
+  <si>
+    <t>e_w799346816-500</t>
+  </si>
+  <si>
+    <t>e_w1016951696-500</t>
+  </si>
+  <si>
+    <t>e_w1373384046-500</t>
+  </si>
+  <si>
+    <t>e_TJ6-500</t>
+  </si>
+  <si>
+    <t>e_TJ29-500</t>
+  </si>
+  <si>
+    <t>e_TJ20-500</t>
+  </si>
+  <si>
+    <t>e_TJ46-500</t>
+  </si>
+  <si>
+    <t>e_TJ30-500</t>
+  </si>
+  <si>
+    <t>e_TJ4-500</t>
+  </si>
+  <si>
+    <t>e_TJ10-500</t>
+  </si>
+  <si>
+    <t>e_TJ26-500</t>
+  </si>
+  <si>
+    <t>elc_spv_001</t>
+  </si>
+  <si>
+    <t>elc_spv_002</t>
+  </si>
+  <si>
+    <t>elc_spv_003</t>
+  </si>
+  <si>
+    <t>elc_spv_004</t>
+  </si>
+  <si>
+    <t>elc_spv_005</t>
+  </si>
+  <si>
+    <t>elc_spv_006</t>
+  </si>
+  <si>
+    <t>elc_spv_007</t>
+  </si>
+  <si>
+    <t>elc_spv_008</t>
+  </si>
+  <si>
+    <t>elc_spv_009</t>
+  </si>
+  <si>
+    <t>elc_spv_010</t>
+  </si>
+  <si>
+    <t>elc_won_001</t>
+  </si>
+  <si>
+    <t>elc_won_002</t>
+  </si>
+  <si>
+    <t>elc_won_003</t>
+  </si>
+  <si>
+    <t>elc_won_004</t>
+  </si>
+  <si>
+    <t>elc_won_005</t>
+  </si>
+  <si>
+    <t>~geolocation</t>
+  </si>
+  <si>
+    <t>region</t>
+  </si>
+  <si>
+    <t>lat</t>
+  </si>
+  <si>
+    <t>lng</t>
+  </si>
+  <si>
+    <t>TJK-e_w242159365-500</t>
+  </si>
+  <si>
+    <t>TJK-e_w488077624-500</t>
+  </si>
+  <si>
+    <t>TJK-e_w799346816-500</t>
+  </si>
+  <si>
+    <t>TJK-e_w1016951696-500</t>
+  </si>
+  <si>
+    <t>TJK-e_w1373384046-500</t>
+  </si>
+  <si>
+    <t>TJK-e_TJ6-500</t>
+  </si>
+  <si>
+    <t>TJK-e_TJ29-500</t>
+  </si>
+  <si>
+    <t>TJK-e_TJ20-500</t>
+  </si>
+  <si>
+    <t>TJK-e_TJ46-500</t>
+  </si>
+  <si>
+    <t>TJK-e_TJ30-500</t>
+  </si>
+  <si>
+    <t>TJK-e_TJ4-500</t>
+  </si>
+  <si>
+    <t>TJK-e_TJ10-500</t>
+  </si>
+  <si>
+    <t>TJK-e_TJ26-500</t>
+  </si>
+  <si>
+    <t>TJK-elc_spv_001</t>
+  </si>
+  <si>
+    <t>TJK-elc_spv_002</t>
+  </si>
+  <si>
+    <t>TJK-elc_spv_003</t>
+  </si>
+  <si>
+    <t>TJK-elc_spv_004</t>
+  </si>
+  <si>
+    <t>TJK-elc_spv_005</t>
+  </si>
+  <si>
+    <t>TJK-elc_spv_006</t>
+  </si>
+  <si>
+    <t>TJK-elc_spv_007</t>
+  </si>
+  <si>
+    <t>TJK-elc_spv_008</t>
+  </si>
+  <si>
+    <t>TJK-elc_spv_009</t>
+  </si>
+  <si>
+    <t>TJK-elc_spv_010</t>
+  </si>
+  <si>
+    <t>TJK-elc_won_001</t>
+  </si>
+  <si>
+    <t>TJK-elc_won_002</t>
+  </si>
+  <si>
+    <t>TJK-elc_won_003</t>
+  </si>
+  <si>
+    <t>TJK-elc_won_004</t>
+  </si>
+  <si>
+    <t>TJK-elc_won_005</t>
   </si>
 </sst>
 </file>
@@ -3925,6 +4236,263 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+  <sheetPr codeName="Sheet2"/>
+  <dimension ref="A1:C13"/>
+  <sheetFormatPr defaultColWidth="9.1328125" defaultRowHeight="14.25"/>
+  <cols>
+    <col min="1" max="1" width="13.59765625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.1328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="36.3984375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" t="s">
+        <v>184</v>
+      </c>
+      <c r="B3" t="str">
+        <f>A3</f>
+        <v>bioenergy</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" t="s">
+        <v>136</v>
+      </c>
+      <c r="B4" t="str">
+        <f t="shared" ref="B4:B11" si="0">A4</f>
+        <v>coal</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" t="s">
+        <v>137</v>
+      </c>
+      <c r="B5" t="str">
+        <f t="shared" si="0"/>
+        <v>gas</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" t="s">
+        <v>265</v>
+      </c>
+      <c r="B6" t="str">
+        <f t="shared" si="0"/>
+        <v>geothermal</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" t="s">
+        <v>266</v>
+      </c>
+      <c r="B7" t="str">
+        <f t="shared" si="0"/>
+        <v>hydro</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" t="s">
+        <v>185</v>
+      </c>
+      <c r="B8" t="str">
+        <f t="shared" si="0"/>
+        <v>hydrogen</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9" t="s">
+        <v>186</v>
+      </c>
+      <c r="B9" t="str">
+        <f t="shared" si="0"/>
+        <v>nuclear</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10" t="s">
+        <v>267</v>
+      </c>
+      <c r="B10" t="str">
+        <f t="shared" si="0"/>
+        <v>oil</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3">
+      <c r="A11" t="s">
+        <v>268</v>
+      </c>
+      <c r="B11" t="str">
+        <f t="shared" si="0"/>
+        <v>solar</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3">
+      <c r="A12" t="s">
+        <v>269</v>
+      </c>
+      <c r="B12" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3">
+      <c r="A13" t="s">
+        <v>270</v>
+      </c>
+      <c r="B13" t="s">
+        <v>272</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32957E82-8232-40A9-A839-CC5F79005B92}">
+  <sheetPr codeName="Sheet3"/>
+  <dimension ref="A1:C10"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col min="1" max="1" width="13.1328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.19921875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.59765625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C2" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" t="s">
+        <v>148</v>
+      </c>
+      <c r="B3" t="s">
+        <v>145</v>
+      </c>
+      <c r="C3" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" t="s">
+        <v>148</v>
+      </c>
+      <c r="B4" t="s">
+        <v>144</v>
+      </c>
+      <c r="C4" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" t="s">
+        <v>149</v>
+      </c>
+      <c r="B5" t="s">
+        <v>150</v>
+      </c>
+      <c r="C5" t="str">
+        <f>LEFT(B5,2)</f>
+        <v>S1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" t="s">
+        <v>149</v>
+      </c>
+      <c r="B6" t="s">
+        <v>151</v>
+      </c>
+      <c r="C6" t="str">
+        <f t="shared" ref="C6:C10" si="0">LEFT(B6,2)</f>
+        <v>S2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" t="s">
+        <v>149</v>
+      </c>
+      <c r="B7" t="s">
+        <v>152</v>
+      </c>
+      <c r="C7" t="str">
+        <f t="shared" si="0"/>
+        <v>S3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" t="s">
+        <v>149</v>
+      </c>
+      <c r="B8" t="s">
+        <v>153</v>
+      </c>
+      <c r="C8" t="str">
+        <f t="shared" si="0"/>
+        <v>S4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9" t="s">
+        <v>149</v>
+      </c>
+      <c r="B9" t="s">
+        <v>154</v>
+      </c>
+      <c r="C9" t="str">
+        <f t="shared" si="0"/>
+        <v>S5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10" t="s">
+        <v>149</v>
+      </c>
+      <c r="B10" t="s">
+        <v>155</v>
+      </c>
+      <c r="C10" t="str">
+        <f t="shared" si="0"/>
+        <v>S6</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{10ADB714-E6AA-4E3E-B77B-62B65BA0E218}">
   <dimension ref="A1:G66"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
@@ -4731,7 +5299,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CE3245E1-8745-41DD-8AE6-2F4FA19D9F1C}">
   <dimension ref="A1:H2"/>
   <sheetFormatPr defaultColWidth="9.1328125" defaultRowHeight="14.25"/>
@@ -4782,7 +5350,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <sheetPr codeName="Sheet4"/>
   <dimension ref="A1:G3"/>
@@ -4827,7 +5395,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <sheetPr codeName="Sheet31"/>
   <dimension ref="A1:D7"/>
@@ -7761,6 +8329,1466 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5AD2FCB1-4E53-4847-8967-719DCE94C87D}">
+  <dimension ref="B9:H38"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetData>
+    <row r="9" spans="2:8">
+      <c r="B9" t="s">
+        <v>494</v>
+      </c>
+      <c r="F9" t="s">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="10" spans="2:8">
+      <c r="B10" t="s">
+        <v>495</v>
+      </c>
+      <c r="C10" t="s">
+        <v>496</v>
+      </c>
+      <c r="D10" t="s">
+        <v>497</v>
+      </c>
+      <c r="F10" t="s">
+        <v>495</v>
+      </c>
+      <c r="G10" t="s">
+        <v>496</v>
+      </c>
+      <c r="H10" t="s">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="11" spans="2:8">
+      <c r="B11" t="s">
+        <v>424</v>
+      </c>
+      <c r="C11">
+        <v>40.113938835875437</v>
+      </c>
+      <c r="D11">
+        <v>69.230840291934925</v>
+      </c>
+      <c r="F11" t="s">
+        <v>498</v>
+      </c>
+      <c r="G11">
+        <v>40.113938835875437</v>
+      </c>
+      <c r="H11">
+        <v>69.230840291934925</v>
+      </c>
+    </row>
+    <row r="12" spans="2:8">
+      <c r="B12" t="s">
+        <v>425</v>
+      </c>
+      <c r="C12">
+        <v>38.553130234478793</v>
+      </c>
+      <c r="D12">
+        <v>68.269751848379315</v>
+      </c>
+      <c r="F12" t="s">
+        <v>499</v>
+      </c>
+      <c r="G12">
+        <v>38.553130234478793</v>
+      </c>
+      <c r="H12">
+        <v>68.269751848379315</v>
+      </c>
+    </row>
+    <row r="13" spans="2:8">
+      <c r="B13" t="s">
+        <v>426</v>
+      </c>
+      <c r="C13">
+        <v>38.67039344075657</v>
+      </c>
+      <c r="D13">
+        <v>69.777117629258683</v>
+      </c>
+      <c r="F13" t="s">
+        <v>500</v>
+      </c>
+      <c r="G13">
+        <v>38.67039344075657</v>
+      </c>
+      <c r="H13">
+        <v>69.777117629258683</v>
+      </c>
+    </row>
+    <row r="14" spans="2:8">
+      <c r="B14" t="s">
+        <v>427</v>
+      </c>
+      <c r="C14">
+        <v>38.381097191055446</v>
+      </c>
+      <c r="D14">
+        <v>69.350268865809227</v>
+      </c>
+      <c r="F14" t="s">
+        <v>501</v>
+      </c>
+      <c r="G14">
+        <v>38.381097191055446</v>
+      </c>
+      <c r="H14">
+        <v>69.350268865809227</v>
+      </c>
+    </row>
+    <row r="15" spans="2:8">
+      <c r="B15" t="s">
+        <v>428</v>
+      </c>
+      <c r="C15">
+        <v>37.944936032738163</v>
+      </c>
+      <c r="D15">
+        <v>69.087985991706802</v>
+      </c>
+      <c r="F15" t="s">
+        <v>502</v>
+      </c>
+      <c r="G15">
+        <v>37.944936032738163</v>
+      </c>
+      <c r="H15">
+        <v>69.087985991706802</v>
+      </c>
+    </row>
+    <row r="16" spans="2:8">
+      <c r="B16" t="s">
+        <v>429</v>
+      </c>
+      <c r="C16">
+        <v>40.578366686872414</v>
+      </c>
+      <c r="D16">
+        <v>69.264023499999979</v>
+      </c>
+      <c r="F16" t="s">
+        <v>503</v>
+      </c>
+      <c r="G16">
+        <v>40.578366686872414</v>
+      </c>
+      <c r="H16">
+        <v>69.264023499999979</v>
+      </c>
+    </row>
+    <row r="17" spans="2:8">
+      <c r="B17" t="s">
+        <v>430</v>
+      </c>
+      <c r="C17">
+        <v>38.693559685045912</v>
+      </c>
+      <c r="D17">
+        <v>66.359086399999981</v>
+      </c>
+      <c r="F17" t="s">
+        <v>504</v>
+      </c>
+      <c r="G17">
+        <v>38.693559685045912</v>
+      </c>
+      <c r="H17">
+        <v>66.359086399999981</v>
+      </c>
+    </row>
+    <row r="18" spans="2:8">
+      <c r="B18" t="s">
+        <v>431</v>
+      </c>
+      <c r="C18">
+        <v>40.222399371237991</v>
+      </c>
+      <c r="D18">
+        <v>69.102056716193772</v>
+      </c>
+      <c r="F18" t="s">
+        <v>505</v>
+      </c>
+      <c r="G18">
+        <v>40.222399371237991</v>
+      </c>
+      <c r="H18">
+        <v>69.102056716193772</v>
+      </c>
+    </row>
+    <row r="19" spans="2:8">
+      <c r="B19" t="s">
+        <v>432</v>
+      </c>
+      <c r="C19">
+        <v>37.521985283865405</v>
+      </c>
+      <c r="D19">
+        <v>67.399013600000004</v>
+      </c>
+      <c r="F19" t="s">
+        <v>506</v>
+      </c>
+      <c r="G19">
+        <v>37.521985283865405</v>
+      </c>
+      <c r="H19">
+        <v>67.399013600000004</v>
+      </c>
+    </row>
+    <row r="20" spans="2:8">
+      <c r="B20" t="s">
+        <v>433</v>
+      </c>
+      <c r="C20">
+        <v>38.673552739925611</v>
+      </c>
+      <c r="D20">
+        <v>68.75452512274353</v>
+      </c>
+      <c r="F20" t="s">
+        <v>507</v>
+      </c>
+      <c r="G20">
+        <v>38.673552739925611</v>
+      </c>
+      <c r="H20">
+        <v>68.75452512274353</v>
+      </c>
+    </row>
+    <row r="21" spans="2:8">
+      <c r="B21" t="s">
+        <v>434</v>
+      </c>
+      <c r="C21">
+        <v>40.713087286998778</v>
+      </c>
+      <c r="D21">
+        <v>69.335133699999957</v>
+      </c>
+      <c r="F21" t="s">
+        <v>508</v>
+      </c>
+      <c r="G21">
+        <v>40.713087286998778</v>
+      </c>
+      <c r="H21">
+        <v>69.335133699999957</v>
+      </c>
+    </row>
+    <row r="22" spans="2:8">
+      <c r="B22" t="s">
+        <v>435</v>
+      </c>
+      <c r="C22">
+        <v>40.3836150866887</v>
+      </c>
+      <c r="D22">
+        <v>70.927240199999986</v>
+      </c>
+      <c r="F22" t="s">
+        <v>509</v>
+      </c>
+      <c r="G22">
+        <v>40.3836150866887</v>
+      </c>
+      <c r="H22">
+        <v>70.927240199999986</v>
+      </c>
+    </row>
+    <row r="23" spans="2:8">
+      <c r="B23" t="s">
+        <v>436</v>
+      </c>
+      <c r="C23">
+        <v>39.930866586256883</v>
+      </c>
+      <c r="D23">
+        <v>69.633654400000012</v>
+      </c>
+      <c r="F23" t="s">
+        <v>510</v>
+      </c>
+      <c r="G23">
+        <v>39.930866586256883</v>
+      </c>
+      <c r="H23">
+        <v>69.633654400000012</v>
+      </c>
+    </row>
+    <row r="24" spans="2:8">
+      <c r="B24" t="s">
+        <v>437</v>
+      </c>
+      <c r="C24">
+        <v>37.620434499878762</v>
+      </c>
+      <c r="D24">
+        <v>71.402194734599803</v>
+      </c>
+      <c r="F24" t="s">
+        <v>511</v>
+      </c>
+      <c r="G24">
+        <v>37.620434499878762</v>
+      </c>
+      <c r="H24">
+        <v>71.402194734599803</v>
+      </c>
+    </row>
+    <row r="25" spans="2:8">
+      <c r="B25" t="s">
+        <v>438</v>
+      </c>
+      <c r="C25">
+        <v>39.64390531825898</v>
+      </c>
+      <c r="D25">
+        <v>71.402194734599803</v>
+      </c>
+      <c r="F25" t="s">
+        <v>512</v>
+      </c>
+      <c r="G25">
+        <v>39.64390531825898</v>
+      </c>
+      <c r="H25">
+        <v>71.402194734599803</v>
+      </c>
+    </row>
+    <row r="26" spans="2:8">
+      <c r="B26" t="s">
+        <v>439</v>
+      </c>
+      <c r="C26">
+        <v>38.086153973950402</v>
+      </c>
+      <c r="D26">
+        <v>69.659774461716708</v>
+      </c>
+      <c r="F26" t="s">
+        <v>513</v>
+      </c>
+      <c r="G26">
+        <v>38.086153973950402</v>
+      </c>
+      <c r="H26">
+        <v>69.659774461716708</v>
+      </c>
+    </row>
+    <row r="27" spans="2:8">
+      <c r="B27" t="s">
+        <v>440</v>
+      </c>
+      <c r="C27">
+        <v>38.1825097272066</v>
+      </c>
+      <c r="D27">
+        <v>68.177715838804673</v>
+      </c>
+      <c r="F27" t="s">
+        <v>514</v>
+      </c>
+      <c r="G27">
+        <v>38.1825097272066</v>
+      </c>
+      <c r="H27">
+        <v>68.177715838804673</v>
+      </c>
+    </row>
+    <row r="28" spans="2:8">
+      <c r="B28" t="s">
+        <v>441</v>
+      </c>
+      <c r="C28">
+        <v>37.283189363482073</v>
+      </c>
+      <c r="D28">
+        <v>69.299273715602979</v>
+      </c>
+      <c r="F28" t="s">
+        <v>515</v>
+      </c>
+      <c r="G28">
+        <v>37.283189363482073</v>
+      </c>
+      <c r="H28">
+        <v>69.299273715602979</v>
+      </c>
+    </row>
+    <row r="29" spans="2:8">
+      <c r="B29" t="s">
+        <v>442</v>
+      </c>
+      <c r="C29">
+        <v>37.283189363482073</v>
+      </c>
+      <c r="D29">
+        <v>68.177715838804673</v>
+      </c>
+      <c r="F29" t="s">
+        <v>516</v>
+      </c>
+      <c r="G29">
+        <v>37.283189363482073</v>
+      </c>
+      <c r="H29">
+        <v>68.177715838804673</v>
+      </c>
+    </row>
+    <row r="30" spans="2:8">
+      <c r="B30" t="s">
+        <v>443</v>
+      </c>
+      <c r="C30">
+        <v>39.231716818218565</v>
+      </c>
+      <c r="D30">
+        <v>70.327368436001422</v>
+      </c>
+      <c r="F30" t="s">
+        <v>517</v>
+      </c>
+      <c r="G30">
+        <v>39.231716818218565</v>
+      </c>
+      <c r="H30">
+        <v>70.327368436001422</v>
+      </c>
+    </row>
+    <row r="31" spans="2:8">
+      <c r="B31" t="s">
+        <v>444</v>
+      </c>
+      <c r="C31">
+        <v>40.430810636517961</v>
+      </c>
+      <c r="D31">
+        <v>69.860052654002132</v>
+      </c>
+      <c r="F31" t="s">
+        <v>518</v>
+      </c>
+      <c r="G31">
+        <v>40.430810636517961</v>
+      </c>
+      <c r="H31">
+        <v>69.860052654002132</v>
+      </c>
+    </row>
+    <row r="32" spans="2:8">
+      <c r="B32" t="s">
+        <v>445</v>
+      </c>
+      <c r="C32">
+        <v>39.756320363724548</v>
+      </c>
+      <c r="D32">
+        <v>68.177715838804673</v>
+      </c>
+      <c r="F32" t="s">
+        <v>519</v>
+      </c>
+      <c r="G32">
+        <v>39.756320363724548</v>
+      </c>
+      <c r="H32">
+        <v>68.177715838804673</v>
+      </c>
+    </row>
+    <row r="33" spans="2:8">
+      <c r="B33" t="s">
+        <v>446</v>
+      </c>
+      <c r="C33">
+        <v>39.306660181862277</v>
+      </c>
+      <c r="D33">
+        <v>69.018884246403402</v>
+      </c>
+      <c r="F33" t="s">
+        <v>520</v>
+      </c>
+      <c r="G33">
+        <v>39.306660181862277</v>
+      </c>
+      <c r="H33">
+        <v>69.018884246403402</v>
+      </c>
+    </row>
+    <row r="34" spans="2:8">
+      <c r="B34" t="s">
+        <v>447</v>
+      </c>
+      <c r="C34">
+        <v>37.058359272550931</v>
+      </c>
+      <c r="D34">
+        <v>67.897326369605111</v>
+      </c>
+      <c r="F34" t="s">
+        <v>521</v>
+      </c>
+      <c r="G34">
+        <v>37.058359272550931</v>
+      </c>
+      <c r="H34">
+        <v>67.897326369605111</v>
+      </c>
+    </row>
+    <row r="35" spans="2:8">
+      <c r="B35" t="s">
+        <v>448</v>
+      </c>
+      <c r="C35">
+        <v>37.058359272550931</v>
+      </c>
+      <c r="D35">
+        <v>68.458105308004249</v>
+      </c>
+      <c r="F35" t="s">
+        <v>522</v>
+      </c>
+      <c r="G35">
+        <v>37.058359272550931</v>
+      </c>
+      <c r="H35">
+        <v>68.458105308004249</v>
+      </c>
+    </row>
+    <row r="36" spans="2:8">
+      <c r="B36" t="s">
+        <v>449</v>
+      </c>
+      <c r="C36">
+        <v>40.655640727449097</v>
+      </c>
+      <c r="D36">
+        <v>69.018884246403402</v>
+      </c>
+      <c r="F36" t="s">
+        <v>523</v>
+      </c>
+      <c r="G36">
+        <v>40.655640727449097</v>
+      </c>
+      <c r="H36">
+        <v>69.018884246403402</v>
+      </c>
+    </row>
+    <row r="37" spans="2:8">
+      <c r="B37" t="s">
+        <v>450</v>
+      </c>
+      <c r="C37">
+        <v>40.655640727449097</v>
+      </c>
+      <c r="D37">
+        <v>69.579663184802556</v>
+      </c>
+      <c r="F37" t="s">
+        <v>524</v>
+      </c>
+      <c r="G37">
+        <v>40.655640727449097</v>
+      </c>
+      <c r="H37">
+        <v>69.579663184802556</v>
+      </c>
+    </row>
+    <row r="38" spans="2:8">
+      <c r="B38" t="s">
+        <v>451</v>
+      </c>
+      <c r="C38">
+        <v>40.655640727449097</v>
+      </c>
+      <c r="D38">
+        <v>70.701221061600862</v>
+      </c>
+      <c r="F38" t="s">
+        <v>525</v>
+      </c>
+      <c r="G38">
+        <v>40.655640727449097</v>
+      </c>
+      <c r="H38">
+        <v>70.701221061600862</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D8FF8D14-B61B-497F-AD95-D295C9C04D44}">
+  <dimension ref="B9:L38"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetData>
+    <row r="9" spans="2:12">
+      <c r="B9" t="s">
+        <v>64</v>
+      </c>
+      <c r="F9" t="s">
+        <v>64</v>
+      </c>
+      <c r="J9" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="10" spans="2:12">
+      <c r="B10" t="s">
+        <v>53</v>
+      </c>
+      <c r="C10" t="s">
+        <v>55</v>
+      </c>
+      <c r="D10" t="s">
+        <v>65</v>
+      </c>
+      <c r="F10" t="s">
+        <v>65</v>
+      </c>
+      <c r="G10" t="s">
+        <v>53</v>
+      </c>
+      <c r="H10" t="s">
+        <v>55</v>
+      </c>
+      <c r="J10" t="s">
+        <v>53</v>
+      </c>
+      <c r="K10" t="s">
+        <v>54</v>
+      </c>
+      <c r="L10" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="11" spans="2:12">
+      <c r="B11" t="s">
+        <v>423</v>
+      </c>
+      <c r="C11" t="s">
+        <v>424</v>
+      </c>
+      <c r="D11" t="s">
+        <v>424</v>
+      </c>
+      <c r="F11" t="s">
+        <v>424</v>
+      </c>
+      <c r="G11" t="s">
+        <v>452</v>
+      </c>
+      <c r="H11" t="s">
+        <v>453</v>
+      </c>
+      <c r="J11" t="s">
+        <v>465</v>
+      </c>
+      <c r="K11" t="s">
+        <v>466</v>
+      </c>
+      <c r="L11" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="12" spans="2:12">
+      <c r="B12" t="s">
+        <v>423</v>
+      </c>
+      <c r="C12" t="s">
+        <v>425</v>
+      </c>
+      <c r="D12" t="s">
+        <v>425</v>
+      </c>
+      <c r="F12" t="s">
+        <v>425</v>
+      </c>
+      <c r="G12" t="s">
+        <v>452</v>
+      </c>
+      <c r="H12" t="s">
+        <v>454</v>
+      </c>
+      <c r="J12" t="s">
+        <v>465</v>
+      </c>
+      <c r="K12" t="s">
+        <v>467</v>
+      </c>
+      <c r="L12" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="13" spans="2:12">
+      <c r="B13" t="s">
+        <v>423</v>
+      </c>
+      <c r="C13" t="s">
+        <v>426</v>
+      </c>
+      <c r="D13" t="s">
+        <v>426</v>
+      </c>
+      <c r="F13" t="s">
+        <v>426</v>
+      </c>
+      <c r="G13" t="s">
+        <v>452</v>
+      </c>
+      <c r="H13" t="s">
+        <v>454</v>
+      </c>
+      <c r="J13" t="s">
+        <v>465</v>
+      </c>
+      <c r="K13" t="s">
+        <v>468</v>
+      </c>
+      <c r="L13" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="14" spans="2:12">
+      <c r="B14" t="s">
+        <v>423</v>
+      </c>
+      <c r="C14" t="s">
+        <v>427</v>
+      </c>
+      <c r="D14" t="s">
+        <v>427</v>
+      </c>
+      <c r="F14" t="s">
+        <v>427</v>
+      </c>
+      <c r="G14" t="s">
+        <v>452</v>
+      </c>
+      <c r="H14" t="s">
+        <v>454</v>
+      </c>
+      <c r="J14" t="s">
+        <v>465</v>
+      </c>
+      <c r="K14" t="s">
+        <v>469</v>
+      </c>
+      <c r="L14" t="s">
+        <v>469</v>
+      </c>
+    </row>
+    <row r="15" spans="2:12">
+      <c r="B15" t="s">
+        <v>423</v>
+      </c>
+      <c r="C15" t="s">
+        <v>428</v>
+      </c>
+      <c r="D15" t="s">
+        <v>428</v>
+      </c>
+      <c r="F15" t="s">
+        <v>428</v>
+      </c>
+      <c r="G15" t="s">
+        <v>452</v>
+      </c>
+      <c r="H15" t="s">
+        <v>455</v>
+      </c>
+      <c r="J15" t="s">
+        <v>465</v>
+      </c>
+      <c r="K15" t="s">
+        <v>470</v>
+      </c>
+      <c r="L15" t="s">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="16" spans="2:12">
+      <c r="B16" t="s">
+        <v>423</v>
+      </c>
+      <c r="C16" t="s">
+        <v>429</v>
+      </c>
+      <c r="D16" t="s">
+        <v>429</v>
+      </c>
+      <c r="F16" t="s">
+        <v>429</v>
+      </c>
+      <c r="G16" t="s">
+        <v>452</v>
+      </c>
+      <c r="H16" t="s">
+        <v>453</v>
+      </c>
+      <c r="J16" t="s">
+        <v>465</v>
+      </c>
+      <c r="K16" t="s">
+        <v>471</v>
+      </c>
+      <c r="L16" t="s">
+        <v>471</v>
+      </c>
+    </row>
+    <row r="17" spans="2:12">
+      <c r="B17" t="s">
+        <v>423</v>
+      </c>
+      <c r="C17" t="s">
+        <v>430</v>
+      </c>
+      <c r="D17" t="s">
+        <v>430</v>
+      </c>
+      <c r="F17" t="s">
+        <v>430</v>
+      </c>
+      <c r="G17" t="s">
+        <v>452</v>
+      </c>
+      <c r="H17" t="s">
+        <v>456</v>
+      </c>
+      <c r="J17" t="s">
+        <v>465</v>
+      </c>
+      <c r="K17" t="s">
+        <v>472</v>
+      </c>
+      <c r="L17" t="s">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="18" spans="2:12">
+      <c r="B18" t="s">
+        <v>423</v>
+      </c>
+      <c r="C18" t="s">
+        <v>431</v>
+      </c>
+      <c r="D18" t="s">
+        <v>431</v>
+      </c>
+      <c r="F18" t="s">
+        <v>431</v>
+      </c>
+      <c r="G18" t="s">
+        <v>452</v>
+      </c>
+      <c r="H18" t="s">
+        <v>457</v>
+      </c>
+      <c r="J18" t="s">
+        <v>465</v>
+      </c>
+      <c r="K18" t="s">
+        <v>473</v>
+      </c>
+      <c r="L18" t="s">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="19" spans="2:12">
+      <c r="B19" t="s">
+        <v>423</v>
+      </c>
+      <c r="C19" t="s">
+        <v>432</v>
+      </c>
+      <c r="D19" t="s">
+        <v>432</v>
+      </c>
+      <c r="F19" t="s">
+        <v>432</v>
+      </c>
+      <c r="G19" t="s">
+        <v>452</v>
+      </c>
+      <c r="H19" t="s">
+        <v>458</v>
+      </c>
+      <c r="J19" t="s">
+        <v>465</v>
+      </c>
+      <c r="K19" t="s">
+        <v>474</v>
+      </c>
+      <c r="L19" t="s">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="20" spans="2:12">
+      <c r="B20" t="s">
+        <v>423</v>
+      </c>
+      <c r="C20" t="s">
+        <v>433</v>
+      </c>
+      <c r="D20" t="s">
+        <v>433</v>
+      </c>
+      <c r="F20" t="s">
+        <v>433</v>
+      </c>
+      <c r="G20" t="s">
+        <v>452</v>
+      </c>
+      <c r="H20" t="s">
+        <v>454</v>
+      </c>
+      <c r="J20" t="s">
+        <v>465</v>
+      </c>
+      <c r="K20" t="s">
+        <v>475</v>
+      </c>
+      <c r="L20" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="21" spans="2:12">
+      <c r="B21" t="s">
+        <v>423</v>
+      </c>
+      <c r="C21" t="s">
+        <v>434</v>
+      </c>
+      <c r="D21" t="s">
+        <v>434</v>
+      </c>
+      <c r="F21" t="s">
+        <v>434</v>
+      </c>
+      <c r="G21" t="s">
+        <v>452</v>
+      </c>
+      <c r="H21" t="s">
+        <v>453</v>
+      </c>
+      <c r="J21" t="s">
+        <v>465</v>
+      </c>
+      <c r="K21" t="s">
+        <v>476</v>
+      </c>
+      <c r="L21" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="22" spans="2:12">
+      <c r="B22" t="s">
+        <v>423</v>
+      </c>
+      <c r="C22" t="s">
+        <v>435</v>
+      </c>
+      <c r="D22" t="s">
+        <v>435</v>
+      </c>
+      <c r="F22" t="s">
+        <v>435</v>
+      </c>
+      <c r="G22" t="s">
+        <v>452</v>
+      </c>
+      <c r="H22" t="s">
+        <v>459</v>
+      </c>
+      <c r="J22" t="s">
+        <v>465</v>
+      </c>
+      <c r="K22" t="s">
+        <v>477</v>
+      </c>
+      <c r="L22" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="23" spans="2:12">
+      <c r="B23" t="s">
+        <v>423</v>
+      </c>
+      <c r="C23" t="s">
+        <v>436</v>
+      </c>
+      <c r="D23" t="s">
+        <v>436</v>
+      </c>
+      <c r="F23" t="s">
+        <v>436</v>
+      </c>
+      <c r="G23" t="s">
+        <v>452</v>
+      </c>
+      <c r="H23" t="s">
+        <v>460</v>
+      </c>
+      <c r="J23" t="s">
+        <v>465</v>
+      </c>
+      <c r="K23" t="s">
+        <v>478</v>
+      </c>
+      <c r="L23" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="24" spans="2:12">
+      <c r="B24" t="s">
+        <v>423</v>
+      </c>
+      <c r="C24" t="s">
+        <v>437</v>
+      </c>
+      <c r="D24" t="s">
+        <v>437</v>
+      </c>
+      <c r="F24" t="s">
+        <v>437</v>
+      </c>
+      <c r="G24" t="s">
+        <v>452</v>
+      </c>
+      <c r="H24" t="s">
+        <v>461</v>
+      </c>
+      <c r="J24" t="s">
+        <v>465</v>
+      </c>
+      <c r="K24" t="s">
+        <v>479</v>
+      </c>
+      <c r="L24" t="s">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="25" spans="2:12">
+      <c r="B25" t="s">
+        <v>423</v>
+      </c>
+      <c r="C25" t="s">
+        <v>438</v>
+      </c>
+      <c r="D25" t="s">
+        <v>438</v>
+      </c>
+      <c r="F25" t="s">
+        <v>438</v>
+      </c>
+      <c r="G25" t="s">
+        <v>452</v>
+      </c>
+      <c r="H25" t="s">
+        <v>460</v>
+      </c>
+      <c r="J25" t="s">
+        <v>465</v>
+      </c>
+      <c r="K25" t="s">
+        <v>480</v>
+      </c>
+      <c r="L25" t="s">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="26" spans="2:12">
+      <c r="B26" t="s">
+        <v>423</v>
+      </c>
+      <c r="C26" t="s">
+        <v>439</v>
+      </c>
+      <c r="D26" t="s">
+        <v>439</v>
+      </c>
+      <c r="F26" t="s">
+        <v>439</v>
+      </c>
+      <c r="G26" t="s">
+        <v>452</v>
+      </c>
+      <c r="H26" t="s">
+        <v>455</v>
+      </c>
+      <c r="J26" t="s">
+        <v>465</v>
+      </c>
+      <c r="K26" t="s">
+        <v>481</v>
+      </c>
+      <c r="L26" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="27" spans="2:12">
+      <c r="B27" t="s">
+        <v>423</v>
+      </c>
+      <c r="C27" t="s">
+        <v>440</v>
+      </c>
+      <c r="D27" t="s">
+        <v>440</v>
+      </c>
+      <c r="F27" t="s">
+        <v>440</v>
+      </c>
+      <c r="G27" t="s">
+        <v>452</v>
+      </c>
+      <c r="H27" t="s">
+        <v>458</v>
+      </c>
+      <c r="J27" t="s">
+        <v>465</v>
+      </c>
+      <c r="K27" t="s">
+        <v>482</v>
+      </c>
+      <c r="L27" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="28" spans="2:12">
+      <c r="B28" t="s">
+        <v>423</v>
+      </c>
+      <c r="C28" t="s">
+        <v>441</v>
+      </c>
+      <c r="D28" t="s">
+        <v>441</v>
+      </c>
+      <c r="F28" t="s">
+        <v>441</v>
+      </c>
+      <c r="G28" t="s">
+        <v>452</v>
+      </c>
+      <c r="H28" t="s">
+        <v>455</v>
+      </c>
+      <c r="J28" t="s">
+        <v>465</v>
+      </c>
+      <c r="K28" t="s">
+        <v>483</v>
+      </c>
+      <c r="L28" t="s">
+        <v>483</v>
+      </c>
+    </row>
+    <row r="29" spans="2:12">
+      <c r="B29" t="s">
+        <v>423</v>
+      </c>
+      <c r="C29" t="s">
+        <v>442</v>
+      </c>
+      <c r="D29" t="s">
+        <v>442</v>
+      </c>
+      <c r="F29" t="s">
+        <v>442</v>
+      </c>
+      <c r="G29" t="s">
+        <v>452</v>
+      </c>
+      <c r="H29" t="s">
+        <v>455</v>
+      </c>
+      <c r="J29" t="s">
+        <v>465</v>
+      </c>
+      <c r="K29" t="s">
+        <v>484</v>
+      </c>
+      <c r="L29" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="30" spans="2:12">
+      <c r="B30" t="s">
+        <v>423</v>
+      </c>
+      <c r="C30" t="s">
+        <v>443</v>
+      </c>
+      <c r="D30" t="s">
+        <v>443</v>
+      </c>
+      <c r="F30" t="s">
+        <v>443</v>
+      </c>
+      <c r="G30" t="s">
+        <v>452</v>
+      </c>
+      <c r="H30" t="s">
+        <v>454</v>
+      </c>
+      <c r="J30" t="s">
+        <v>465</v>
+      </c>
+      <c r="K30" t="s">
+        <v>485</v>
+      </c>
+      <c r="L30" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="31" spans="2:12">
+      <c r="B31" t="s">
+        <v>423</v>
+      </c>
+      <c r="C31" t="s">
+        <v>444</v>
+      </c>
+      <c r="D31" t="s">
+        <v>444</v>
+      </c>
+      <c r="F31" t="s">
+        <v>444</v>
+      </c>
+      <c r="G31" t="s">
+        <v>452</v>
+      </c>
+      <c r="H31" t="s">
+        <v>453</v>
+      </c>
+      <c r="J31" t="s">
+        <v>465</v>
+      </c>
+      <c r="K31" t="s">
+        <v>486</v>
+      </c>
+      <c r="L31" t="s">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="32" spans="2:12">
+      <c r="B32" t="s">
+        <v>423</v>
+      </c>
+      <c r="C32" t="s">
+        <v>445</v>
+      </c>
+      <c r="D32" t="s">
+        <v>445</v>
+      </c>
+      <c r="F32" t="s">
+        <v>445</v>
+      </c>
+      <c r="G32" t="s">
+        <v>452</v>
+      </c>
+      <c r="H32" t="s">
+        <v>462</v>
+      </c>
+      <c r="J32" t="s">
+        <v>465</v>
+      </c>
+      <c r="K32" t="s">
+        <v>487</v>
+      </c>
+      <c r="L32" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="33" spans="2:12">
+      <c r="B33" t="s">
+        <v>423</v>
+      </c>
+      <c r="C33" t="s">
+        <v>446</v>
+      </c>
+      <c r="D33" t="s">
+        <v>446</v>
+      </c>
+      <c r="F33" t="s">
+        <v>446</v>
+      </c>
+      <c r="G33" t="s">
+        <v>452</v>
+      </c>
+      <c r="H33" t="s">
+        <v>453</v>
+      </c>
+      <c r="J33" t="s">
+        <v>465</v>
+      </c>
+      <c r="K33" t="s">
+        <v>488</v>
+      </c>
+      <c r="L33" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="34" spans="2:12">
+      <c r="B34" t="s">
+        <v>423</v>
+      </c>
+      <c r="C34" t="s">
+        <v>447</v>
+      </c>
+      <c r="D34" t="s">
+        <v>447</v>
+      </c>
+      <c r="F34" t="s">
+        <v>447</v>
+      </c>
+      <c r="G34" t="s">
+        <v>452</v>
+      </c>
+      <c r="H34" t="s">
+        <v>455</v>
+      </c>
+      <c r="J34" t="s">
+        <v>465</v>
+      </c>
+      <c r="K34" t="s">
+        <v>489</v>
+      </c>
+      <c r="L34" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="35" spans="2:12">
+      <c r="B35" t="s">
+        <v>423</v>
+      </c>
+      <c r="C35" t="s">
+        <v>448</v>
+      </c>
+      <c r="D35" t="s">
+        <v>448</v>
+      </c>
+      <c r="F35" t="s">
+        <v>448</v>
+      </c>
+      <c r="G35" t="s">
+        <v>452</v>
+      </c>
+      <c r="H35" t="s">
+        <v>463</v>
+      </c>
+      <c r="J35" t="s">
+        <v>465</v>
+      </c>
+      <c r="K35" t="s">
+        <v>490</v>
+      </c>
+      <c r="L35" t="s">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="36" spans="2:12">
+      <c r="B36" t="s">
+        <v>423</v>
+      </c>
+      <c r="C36" t="s">
+        <v>449</v>
+      </c>
+      <c r="D36" t="s">
+        <v>449</v>
+      </c>
+      <c r="F36" t="s">
+        <v>449</v>
+      </c>
+      <c r="G36" t="s">
+        <v>452</v>
+      </c>
+      <c r="H36" t="s">
+        <v>464</v>
+      </c>
+      <c r="J36" t="s">
+        <v>465</v>
+      </c>
+      <c r="K36" t="s">
+        <v>491</v>
+      </c>
+      <c r="L36" t="s">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="37" spans="2:12">
+      <c r="B37" t="s">
+        <v>423</v>
+      </c>
+      <c r="C37" t="s">
+        <v>450</v>
+      </c>
+      <c r="D37" t="s">
+        <v>450</v>
+      </c>
+      <c r="F37" t="s">
+        <v>450</v>
+      </c>
+      <c r="G37" t="s">
+        <v>452</v>
+      </c>
+      <c r="H37" t="s">
+        <v>453</v>
+      </c>
+      <c r="J37" t="s">
+        <v>465</v>
+      </c>
+      <c r="K37" t="s">
+        <v>492</v>
+      </c>
+      <c r="L37" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="38" spans="2:12">
+      <c r="B38" t="s">
+        <v>423</v>
+      </c>
+      <c r="C38" t="s">
+        <v>451</v>
+      </c>
+      <c r="D38" t="s">
+        <v>451</v>
+      </c>
+      <c r="F38" t="s">
+        <v>451</v>
+      </c>
+      <c r="G38" t="s">
+        <v>452</v>
+      </c>
+      <c r="H38" t="s">
+        <v>459</v>
+      </c>
+      <c r="J38" t="s">
+        <v>465</v>
+      </c>
+      <c r="K38" t="s">
+        <v>493</v>
+      </c>
+      <c r="L38" t="s">
+        <v>493</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet19"/>
   <dimension ref="A1:U22"/>
@@ -8238,7 +10266,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68A8EC7F-95E3-4526-8B78-C58A96098159}">
   <dimension ref="C1:K3"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
@@ -8318,7 +10346,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{31D44EBE-400A-4EA2-9DA1-076783A77DFC}">
   <dimension ref="A3:S23"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
@@ -8677,7 +10705,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:C47"/>
@@ -9113,7 +11141,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A3E766D8-7F73-4A5A-98A5-9C85D527817F}">
   <dimension ref="A1:C35"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
@@ -9429,263 +11457,6 @@
       <c r="B35" s="7" t="str">
         <f t="shared" si="2"/>
         <v>nuclear</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <sheetPr codeName="Sheet2"/>
-  <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultColWidth="9.1328125" defaultRowHeight="14.25"/>
-  <cols>
-    <col min="1" max="1" width="13.59765625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.1328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="36.3984375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3">
-      <c r="A1" s="1" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="A2" t="s">
-        <v>28</v>
-      </c>
-      <c r="B2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
-      <c r="A3" t="s">
-        <v>184</v>
-      </c>
-      <c r="B3" t="str">
-        <f>A3</f>
-        <v>bioenergy</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3">
-      <c r="A4" t="s">
-        <v>136</v>
-      </c>
-      <c r="B4" t="str">
-        <f t="shared" ref="B4:B11" si="0">A4</f>
-        <v>coal</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3">
-      <c r="A5" t="s">
-        <v>137</v>
-      </c>
-      <c r="B5" t="str">
-        <f t="shared" si="0"/>
-        <v>gas</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3">
-      <c r="A6" t="s">
-        <v>265</v>
-      </c>
-      <c r="B6" t="str">
-        <f t="shared" si="0"/>
-        <v>geothermal</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3">
-      <c r="A7" t="s">
-        <v>266</v>
-      </c>
-      <c r="B7" t="str">
-        <f t="shared" si="0"/>
-        <v>hydro</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3">
-      <c r="A8" t="s">
-        <v>185</v>
-      </c>
-      <c r="B8" t="str">
-        <f t="shared" si="0"/>
-        <v>hydrogen</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3">
-      <c r="A9" t="s">
-        <v>186</v>
-      </c>
-      <c r="B9" t="str">
-        <f t="shared" si="0"/>
-        <v>nuclear</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3">
-      <c r="A10" t="s">
-        <v>267</v>
-      </c>
-      <c r="B10" t="str">
-        <f t="shared" si="0"/>
-        <v>oil</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3">
-      <c r="A11" t="s">
-        <v>268</v>
-      </c>
-      <c r="B11" t="str">
-        <f t="shared" si="0"/>
-        <v>solar</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3">
-      <c r="A12" t="s">
-        <v>269</v>
-      </c>
-      <c r="B12" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3">
-      <c r="A13" t="s">
-        <v>270</v>
-      </c>
-      <c r="B13" t="s">
-        <v>272</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32957E82-8232-40A9-A839-CC5F79005B92}">
-  <sheetPr codeName="Sheet3"/>
-  <dimension ref="A1:C10"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
-  <cols>
-    <col min="1" max="1" width="13.1328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.19921875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.59765625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3">
-      <c r="A1" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="A2" t="s">
-        <v>53</v>
-      </c>
-      <c r="B2" t="s">
-        <v>54</v>
-      </c>
-      <c r="C2" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
-      <c r="A3" t="s">
-        <v>148</v>
-      </c>
-      <c r="B3" t="s">
-        <v>145</v>
-      </c>
-      <c r="C3" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3">
-      <c r="A4" t="s">
-        <v>148</v>
-      </c>
-      <c r="B4" t="s">
-        <v>144</v>
-      </c>
-      <c r="C4" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3">
-      <c r="A5" t="s">
-        <v>149</v>
-      </c>
-      <c r="B5" t="s">
-        <v>150</v>
-      </c>
-      <c r="C5" t="str">
-        <f>LEFT(B5,2)</f>
-        <v>S1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3">
-      <c r="A6" t="s">
-        <v>149</v>
-      </c>
-      <c r="B6" t="s">
-        <v>151</v>
-      </c>
-      <c r="C6" t="str">
-        <f t="shared" ref="C6:C10" si="0">LEFT(B6,2)</f>
-        <v>S2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3">
-      <c r="A7" t="s">
-        <v>149</v>
-      </c>
-      <c r="B7" t="s">
-        <v>152</v>
-      </c>
-      <c r="C7" t="str">
-        <f t="shared" si="0"/>
-        <v>S3</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3">
-      <c r="A8" t="s">
-        <v>149</v>
-      </c>
-      <c r="B8" t="s">
-        <v>153</v>
-      </c>
-      <c r="C8" t="str">
-        <f t="shared" si="0"/>
-        <v>S4</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3">
-      <c r="A9" t="s">
-        <v>149</v>
-      </c>
-      <c r="B9" t="s">
-        <v>154</v>
-      </c>
-      <c r="C9" t="str">
-        <f t="shared" si="0"/>
-        <v>S5</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3">
-      <c r="A10" t="s">
-        <v>149</v>
-      </c>
-      <c r="B10" t="s">
-        <v>155</v>
-      </c>
-      <c r="C10" t="str">
-        <f t="shared" si="0"/>
-        <v>S6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>